<commit_message>
puntaje estimado de nota con lo que hay ~60
</commit_message>
<xml_diff>
--- a/Rubrica_Caso_BD.xlsx
+++ b/Rubrica_Caso_BD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\USM\AyudantiaBD\2026-1\t3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\caso_BD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4771A000-3BED-4A88-8102-88205AE4733A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2FBD014-29D8-4275-A44B-E753C328CFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rúbrica" sheetId="1" r:id="rId1"/>
@@ -739,7 +739,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
@@ -751,7 +751,7 @@
     <col min="13" max="14" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="17" t="s">
         <v>103</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="J1" s="15"/>
       <c r="K1" s="15"/>
     </row>
-    <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>0</v>
       </c>
@@ -781,7 +781,7 @@
       <c r="J2" s="15"/>
       <c r="K2" s="15"/>
     </row>
-    <row r="4" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>1</v>
       </c>
@@ -789,7 +789,7 @@
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
     </row>
-    <row r="5" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -809,7 +809,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -829,7 +829,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -849,7 +849,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
@@ -869,7 +869,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -889,7 +889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -909,7 +909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>22</v>
       </c>
@@ -924,7 +924,7 @@
       <c r="J11" s="15"/>
       <c r="K11" s="15"/>
     </row>
-    <row r="12" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>23</v>
       </c>
@@ -959,7 +959,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>1</v>
       </c>
@@ -985,13 +985,12 @@
         <v>35</v>
       </c>
       <c r="I13" s="2"/>
-      <c r="J13" s="2" t="str">
-        <f t="shared" ref="J13:J21" si="0">IF(I13="","",VLOOKUP(I13,$M$6:$N$10,2,FALSE))</f>
-        <v/>
+      <c r="J13" s="2">
+        <v>6</v>
       </c>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>2</v>
       </c>
@@ -1017,13 +1016,12 @@
         <v>41</v>
       </c>
       <c r="I14" s="2"/>
-      <c r="J14" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J14" s="2">
+        <v>6</v>
       </c>
       <c r="K14" s="3"/>
     </row>
-    <row r="15" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>3</v>
       </c>
@@ -1049,13 +1047,12 @@
         <v>47</v>
       </c>
       <c r="I15" s="2"/>
-      <c r="J15" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J15" s="2">
+        <v>6</v>
       </c>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>4</v>
       </c>
@@ -1081,13 +1078,12 @@
         <v>53</v>
       </c>
       <c r="I16" s="2"/>
-      <c r="J16" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J16" s="2">
+        <v>6</v>
       </c>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>5</v>
       </c>
@@ -1113,13 +1109,12 @@
         <v>59</v>
       </c>
       <c r="I17" s="2"/>
-      <c r="J17" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J17" s="2">
+        <v>6</v>
       </c>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>6</v>
       </c>
@@ -1145,13 +1140,12 @@
         <v>65</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="J18" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J18" s="2">
+        <v>6</v>
       </c>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>7</v>
       </c>
@@ -1177,13 +1171,12 @@
         <v>71</v>
       </c>
       <c r="I19" s="2"/>
-      <c r="J19" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J19" s="2">
+        <v>6</v>
       </c>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>8</v>
       </c>
@@ -1209,13 +1202,12 @@
         <v>77</v>
       </c>
       <c r="I20" s="2"/>
-      <c r="J20" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J20" s="2">
+        <v>6</v>
       </c>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>9</v>
       </c>
@@ -1241,13 +1233,12 @@
         <v>83</v>
       </c>
       <c r="I21" s="2"/>
-      <c r="J21" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+      <c r="J21" s="2">
+        <v>0</v>
       </c>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="5"/>
       <c r="C22" s="4"/>
@@ -1261,11 +1252,11 @@
       </c>
       <c r="J22" s="6">
         <f>SUM(J13:J21)</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="K22" s="5"/>
     </row>
-    <row r="23" spans="1:11" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -1296,7 +1287,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>10</v>
       </c>
@@ -1318,10 +1309,12 @@
       </c>
       <c r="H24" s="3"/>
       <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
+      <c r="J24" s="2">
+        <v>4</v>
+      </c>
       <c r="K24" s="3"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>11</v>
       </c>
@@ -1343,10 +1336,12 @@
       </c>
       <c r="H25" s="3"/>
       <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
+      <c r="J25" s="2">
+        <v>4</v>
+      </c>
       <c r="K25" s="3"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>12</v>
       </c>
@@ -1368,10 +1363,12 @@
       </c>
       <c r="H26" s="3"/>
       <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
+      <c r="J26" s="2">
+        <v>4</v>
+      </c>
       <c r="K26" s="3"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>13</v>
       </c>
@@ -1392,10 +1389,12 @@
         <v>0</v>
       </c>
       <c r="H27" s="3"/>
-      <c r="J27" s="10"/>
+      <c r="J27" s="10">
+        <v>4</v>
+      </c>
       <c r="K27" s="3"/>
     </row>
-    <row r="28" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -1409,11 +1408,11 @@
       </c>
       <c r="J28" s="6">
         <f>SUM(J24:J27)</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="K28" s="5"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1426,7 +1425,7 @@
       <c r="J29" s="12"/>
       <c r="K29" s="11"/>
     </row>
-    <row r="30" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
         <v>85</v>
       </c>
@@ -1434,7 +1433,7 @@
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
       <c r="B31" s="5" t="s">
         <v>86</v>
@@ -1443,7 +1442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="5"/>
       <c r="B32" s="5" t="s">
         <v>87</v>
@@ -1452,7 +1451,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="5"/>
       <c r="B33" s="5" t="s">
         <v>88</v>
@@ -1461,24 +1460,24 @@
         <v>89</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="5"/>
       <c r="B34" s="5" t="s">
         <v>90</v>
       </c>
       <c r="C34" s="5">
         <f>IF(C33="NO",0,MAX(0,MIN(100,J22+J28 - IF(C31&gt;0,CEILING(C31,1)*C32,0))))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="5"/>
       <c r="B35" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C35" s="5" t="str">
         <f>IF(C34&gt;=55,"APROBADO","REPROBADO")</f>
-        <v>REPROBADO</v>
+        <v>APROBADO</v>
       </c>
     </row>
   </sheetData>
@@ -1505,147 +1504,147 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="9"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="9"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="9"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="9"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="9"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="9"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="9"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="9"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="9"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="9"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="9"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="9"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="9"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="9"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="9"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="9"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="9"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="9"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="9"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="9"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="9"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="9"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="9"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="9"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="9"/>
     </row>
   </sheetData>

</xml_diff>